<commit_message>
Cambios en el remito. Mas lineas y menos margen
</commit_message>
<xml_diff>
--- a/DOCS/REMITO_Master.xlsx
+++ b/DOCS/REMITO_Master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORKS\CAPELLO SOMBREROS\APPLICATION\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F4D1D0-9D95-499F-8D70-ECA5EC1B0B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7C1231-3F4B-458A-932A-42835517CB50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Remito" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Remito!$A$1:$H$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Remito!$A$1:$H$52</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -189,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -348,17 +348,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top/>
       <bottom style="thin">
@@ -372,7 +361,7 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -488,9 +477,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -500,10 +486,24 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -525,21 +525,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -848,7 +833,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:AR857"/>
+  <dimension ref="A1:AR861"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.109375" customWidth="1"/>
@@ -870,30 +855,30 @@
       <c r="H1" s="10"/>
     </row>
     <row r="2" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="1.05">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="67" t="s">
+      <c r="B2"/>
+      <c r="C2" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="69">
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="55">
         <v>0.7</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="63"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="64"/>
+      <c r="A3" s="56"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="51"/>
     </row>
     <row r="4" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="23"/>
@@ -906,28 +891,28 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="58"/>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="55" t="s">
+      <c r="A5" s="63"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="52"/>
+      <c r="G5" s="60"/>
       <c r="H5" s="37"/>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="60"/>
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="57"/>
+      <c r="A6" s="65"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="62"/>
       <c r="F6" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="56"/>
-      <c r="H6" s="57"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="62"/>
     </row>
     <row r="7" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="23"/>
@@ -940,16 +925,16 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="61" t="s">
+      <c r="A8" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="G8" s="62"/>
-      <c r="H8" s="51" t="s">
+      <c r="B8" s="67"/>
+      <c r="C8" s="67"/>
+      <c r="D8" s="67"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="67"/>
+      <c r="G8" s="67"/>
+      <c r="H8" s="50" t="s">
         <v>21</v>
       </c>
     </row>
@@ -984,11 +969,11 @@
     <row r="10" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="31"/>
       <c r="B10" s="24"/>
-      <c r="C10" s="49" t="str">
+      <c r="C10" s="48" t="str">
         <f>IF(D10 ="","",D10*$H$2)</f>
         <v/>
       </c>
-      <c r="D10" s="49"/>
+      <c r="D10" s="48"/>
       <c r="E10" s="31"/>
       <c r="F10" s="38"/>
       <c r="G10" s="38"/>
@@ -997,11 +982,11 @@
     <row r="11" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="32"/>
       <c r="B11" s="24"/>
-      <c r="C11" s="49" t="str">
-        <f t="shared" ref="C11:C34" si="0">IF(D11 ="","",D11*$H$2)</f>
-        <v/>
-      </c>
-      <c r="D11" s="49"/>
+      <c r="C11" s="48" t="str">
+        <f t="shared" ref="C11:C38" si="0">IF(D11 ="","",D11*$H$2)</f>
+        <v/>
+      </c>
+      <c r="D11" s="48"/>
       <c r="E11" s="32"/>
       <c r="F11" s="39"/>
       <c r="G11" s="39"/>
@@ -1010,11 +995,11 @@
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="33"/>
       <c r="B12" s="24"/>
-      <c r="C12" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D12" s="49"/>
+      <c r="C12" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D12" s="48"/>
       <c r="E12" s="40"/>
       <c r="F12" s="41"/>
       <c r="G12" s="42"/>
@@ -1023,11 +1008,11 @@
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="31"/>
       <c r="B13" s="24"/>
-      <c r="C13" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D13" s="49"/>
+      <c r="C13" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D13" s="48"/>
       <c r="E13" s="31"/>
       <c r="F13" s="36"/>
       <c r="G13" s="36"/>
@@ -1036,11 +1021,11 @@
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="31"/>
       <c r="B14" s="24"/>
-      <c r="C14" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D14" s="49"/>
+      <c r="C14" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D14" s="48"/>
       <c r="E14" s="31"/>
       <c r="F14" s="43"/>
       <c r="G14" s="43"/>
@@ -1049,11 +1034,11 @@
     <row r="15" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="31"/>
       <c r="B15" s="24"/>
-      <c r="C15" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D15" s="49"/>
+      <c r="C15" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D15" s="48"/>
       <c r="E15" s="31"/>
       <c r="F15" s="38"/>
       <c r="G15" s="38"/>
@@ -1062,129 +1047,117 @@
     <row r="16" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="31"/>
       <c r="B16" s="24"/>
-      <c r="C16" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D16" s="49"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="48"/>
       <c r="E16" s="31"/>
       <c r="F16" s="38"/>
       <c r="G16" s="38"/>
-      <c r="H16" s="45"/>
+      <c r="H16" s="39"/>
     </row>
     <row r="17" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="31"/>
       <c r="B17" s="24"/>
-      <c r="C17" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D17" s="49"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="48"/>
       <c r="E17" s="31"/>
       <c r="F17" s="38"/>
       <c r="G17" s="38"/>
-      <c r="H17" s="48"/>
+      <c r="H17" s="39"/>
     </row>
     <row r="18" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="31"/>
       <c r="B18" s="24"/>
-      <c r="C18" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D18" s="49"/>
+      <c r="C18" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D18" s="48"/>
       <c r="E18" s="31"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="45"/>
     </row>
     <row r="19" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="24"/>
-      <c r="C19" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D19" s="49"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="44"/>
-      <c r="G19" s="44"/>
-      <c r="H19" s="39"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="34"/>
+      <c r="C19" s="48"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="48"/>
+    </row>
+    <row r="20" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="31"/>
       <c r="B20" s="24"/>
-      <c r="C20" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D20" s="49"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="45"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="38"/>
+      <c r="H20" s="48"/>
     </row>
     <row r="21" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="31"/>
       <c r="B21" s="24"/>
-      <c r="C21" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D21" s="49"/>
+      <c r="C21" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D21" s="48"/>
       <c r="E21" s="31"/>
       <c r="F21" s="38"/>
       <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
+      <c r="H21" s="48"/>
     </row>
     <row r="22" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
+      <c r="A22" s="31"/>
       <c r="B22" s="24"/>
-      <c r="C22" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D22" s="49"/>
-      <c r="E22" s="32"/>
+      <c r="C22" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D22" s="48"/>
+      <c r="E22" s="31"/>
       <c r="F22" s="39"/>
       <c r="G22" s="39"/>
       <c r="H22" s="39"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="35"/>
+    <row r="23" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="34"/>
       <c r="B23" s="24"/>
-      <c r="C23" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D23" s="49"/>
+      <c r="C23" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D23" s="48"/>
       <c r="E23" s="32"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="41"/>
-    </row>
-    <row r="24" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="31"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="39"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="34"/>
       <c r="B24" s="24"/>
-      <c r="C24" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D24" s="49"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="38"/>
+      <c r="C24" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D24" s="48"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="45"/>
     </row>
     <row r="25" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="31"/>
       <c r="B25" s="24"/>
-      <c r="C25" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D25" s="49"/>
-      <c r="E25" s="32"/>
+      <c r="C25" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D25" s="48"/>
+      <c r="E25" s="31"/>
       <c r="F25" s="38"/>
       <c r="G25" s="38"/>
       <c r="H25" s="38"/>
@@ -1192,37 +1165,37 @@
     <row r="26" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="32"/>
       <c r="B26" s="24"/>
-      <c r="C26" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D26" s="49"/>
-      <c r="E26" s="46"/>
+      <c r="C26" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D26" s="48"/>
+      <c r="E26" s="32"/>
       <c r="F26" s="39"/>
       <c r="G26" s="39"/>
       <c r="H26" s="39"/>
     </row>
-    <row r="27" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="31"/>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="35"/>
       <c r="B27" s="24"/>
-      <c r="C27" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D27" s="49"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="38"/>
+      <c r="C27" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D27" s="48"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="41"/>
     </row>
     <row r="28" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="31"/>
       <c r="B28" s="24"/>
-      <c r="C28" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D28" s="49"/>
+      <c r="C28" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D28" s="48"/>
       <c r="E28" s="31"/>
       <c r="F28" s="38"/>
       <c r="G28" s="38"/>
@@ -1231,37 +1204,37 @@
     <row r="29" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="31"/>
       <c r="B29" s="24"/>
-      <c r="C29" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D29" s="49"/>
-      <c r="E29" s="31"/>
+      <c r="C29" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D29" s="48"/>
+      <c r="E29" s="32"/>
       <c r="F29" s="38"/>
       <c r="G29" s="38"/>
       <c r="H29" s="38"/>
     </row>
     <row r="30" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="31"/>
+      <c r="A30" s="32"/>
       <c r="B30" s="24"/>
-      <c r="C30" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D30" s="49"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="38"/>
-      <c r="H30" s="38"/>
+      <c r="C30" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D30" s="48"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="39"/>
     </row>
     <row r="31" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="31"/>
       <c r="B31" s="24"/>
-      <c r="C31" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D31" s="49"/>
+      <c r="C31" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D31" s="48"/>
       <c r="E31" s="31"/>
       <c r="F31" s="38"/>
       <c r="G31" s="38"/>
@@ -1270,11 +1243,11 @@
     <row r="32" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="31"/>
       <c r="B32" s="24"/>
-      <c r="C32" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D32" s="49"/>
+      <c r="C32" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D32" s="48"/>
       <c r="E32" s="31"/>
       <c r="F32" s="38"/>
       <c r="G32" s="38"/>
@@ -1283,152 +1256,160 @@
     <row r="33" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="31"/>
       <c r="B33" s="24"/>
-      <c r="C33" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D33" s="49"/>
+      <c r="C33" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D33" s="48"/>
       <c r="E33" s="31"/>
       <c r="F33" s="38"/>
       <c r="G33" s="38"/>
       <c r="H33" s="38"/>
     </row>
-    <row r="34" spans="1:44" s="26" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="32"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="50" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D34" s="50"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="H34" s="39"/>
-      <c r="I34"/>
-      <c r="J34"/>
-      <c r="K34"/>
-      <c r="L34"/>
-      <c r="M34"/>
-      <c r="N34"/>
-      <c r="O34"/>
-      <c r="P34"/>
-      <c r="Q34"/>
-      <c r="R34"/>
-      <c r="S34"/>
-      <c r="T34"/>
-      <c r="U34"/>
-      <c r="V34"/>
-      <c r="W34"/>
-      <c r="X34"/>
-      <c r="Y34"/>
-      <c r="Z34"/>
-      <c r="AA34"/>
-      <c r="AB34"/>
-      <c r="AC34"/>
-      <c r="AD34"/>
-      <c r="AE34"/>
-      <c r="AF34"/>
-      <c r="AG34"/>
-      <c r="AH34"/>
-      <c r="AI34"/>
-      <c r="AJ34"/>
-      <c r="AK34"/>
-      <c r="AL34"/>
-      <c r="AM34"/>
-      <c r="AN34"/>
-      <c r="AO34"/>
-      <c r="AP34"/>
-      <c r="AQ34"/>
-      <c r="AR34"/>
-    </row>
-    <row r="35" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A35" s="19"/>
-      <c r="C35" t="s">
+    <row r="34" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="31"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D34" s="48"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+    </row>
+    <row r="35" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="31"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D35" s="48"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+    </row>
+    <row r="36" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="31"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D36" s="48"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+    </row>
+    <row r="37" spans="1:44" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="31"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D37" s="48"/>
+      <c r="E37" s="31"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+    </row>
+    <row r="38" spans="1:44" s="26" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="32"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D38" s="49"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="39"/>
+      <c r="I38"/>
+      <c r="J38"/>
+      <c r="K38"/>
+      <c r="L38"/>
+      <c r="M38"/>
+      <c r="N38"/>
+      <c r="O38"/>
+      <c r="P38"/>
+      <c r="Q38"/>
+      <c r="R38"/>
+      <c r="S38"/>
+      <c r="T38"/>
+      <c r="U38"/>
+      <c r="V38"/>
+      <c r="W38"/>
+      <c r="X38"/>
+      <c r="Y38"/>
+      <c r="Z38"/>
+      <c r="AA38"/>
+      <c r="AB38"/>
+      <c r="AC38"/>
+      <c r="AD38"/>
+      <c r="AE38"/>
+      <c r="AF38"/>
+      <c r="AG38"/>
+      <c r="AH38"/>
+      <c r="AI38"/>
+      <c r="AJ38"/>
+      <c r="AK38"/>
+      <c r="AL38"/>
+      <c r="AM38"/>
+      <c r="AN38"/>
+      <c r="AO38"/>
+      <c r="AP38"/>
+      <c r="AQ38"/>
+      <c r="AR38"/>
+    </row>
+    <row r="39" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A39" s="19"/>
+      <c r="C39" t="s">
         <v>15</v>
       </c>
-      <c r="D35" s="5"/>
-      <c r="E35" s="40">
-        <f>SUM(E10:E34)</f>
+      <c r="D39" s="5"/>
+      <c r="E39" s="40">
+        <f>SUM(E10:E38)</f>
         <v>0</v>
       </c>
-      <c r="H35" s="12"/>
-    </row>
-    <row r="36" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A36" s="11"/>
-      <c r="B36" s="18"/>
-      <c r="C36" t="s">
-        <v>16</v>
-      </c>
-      <c r="D36" s="5"/>
-      <c r="E36" s="40">
-        <f>SUM(F10:F34)</f>
-        <v>0</v>
-      </c>
-      <c r="H36" s="25"/>
-    </row>
-    <row r="37" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A37" s="11"/>
-      <c r="B37" s="18"/>
-      <c r="C37" t="s">
-        <v>17</v>
-      </c>
-      <c r="D37" s="5"/>
-      <c r="E37" s="40">
-        <f>SUM(G10:G34)</f>
-        <v>0</v>
-      </c>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="25"/>
-    </row>
-    <row r="38" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A38" s="11"/>
-      <c r="B38" s="18"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="5"/>
-    </row>
-    <row r="39" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A39" s="11"/>
-      <c r="B39" s="18"/>
-      <c r="C39" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D39" s="6"/>
-      <c r="E39" s="20"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="7"/>
+      <c r="H39" s="12"/>
     </row>
     <row r="40" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A40" s="11"/>
       <c r="B40" s="18"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
-      <c r="H40" s="5"/>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40" s="5"/>
+      <c r="E40" s="40">
+        <f>SUM(F10:F38)</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="25"/>
     </row>
     <row r="41" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A41" s="11"/>
       <c r="B41" s="18"/>
-      <c r="C41" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D41" s="6"/>
-      <c r="E41" s="20"/>
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="7"/>
+      <c r="C41" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" s="5"/>
+      <c r="E41" s="40">
+        <f>SUM(G10:G38)</f>
+        <v>0</v>
+      </c>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="25"/>
     </row>
     <row r="42" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A42" s="11"/>
       <c r="B42" s="18"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="18"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="5"/>
@@ -1437,16 +1418,16 @@
       <c r="A43" s="11"/>
       <c r="B43" s="18"/>
       <c r="C43" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D43" s="53"/>
-      <c r="E43" s="54"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
-      <c r="H43" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="D43" s="6"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="7"/>
     </row>
     <row r="44" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A44" s="22"/>
+      <c r="A44" s="11"/>
       <c r="B44" s="18"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
@@ -1458,40 +1439,40 @@
     <row r="45" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A45" s="11"/>
       <c r="B45" s="18"/>
-      <c r="C45" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D45" s="1"/>
-      <c r="E45" s="47"/>
-      <c r="F45" s="47"/>
-      <c r="G45" s="47"/>
-      <c r="H45" s="5"/>
+      <c r="C45" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D45" s="6"/>
+      <c r="E45" s="20"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="6"/>
+      <c r="H45" s="7"/>
     </row>
     <row r="46" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A46" s="11"/>
       <c r="B46" s="18"/>
-      <c r="C46" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="C46" s="1"/>
       <c r="D46" s="1"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="47"/>
-      <c r="G46" s="47"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
       <c r="H46" s="5"/>
     </row>
     <row r="47" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A47" s="11"/>
-      <c r="B47" s="1"/>
-      <c r="C47" s="1"/>
-      <c r="D47" s="1"/>
-      <c r="E47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D47" s="58"/>
+      <c r="E47" s="57"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="5"/>
     </row>
     <row r="48" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A48" s="11"/>
-      <c r="B48" s="1"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="18"/>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
       <c r="E48" s="18"/>
@@ -1499,8 +1480,52 @@
       <c r="G48" s="1"/>
       <c r="H48" s="5"/>
     </row>
-    <row r="857" spans="10:10" x14ac:dyDescent="0.25">
-      <c r="J857" t="s">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="11"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D49" s="1"/>
+      <c r="E49" s="47"/>
+      <c r="F49" s="47"/>
+      <c r="G49" s="47"/>
+      <c r="H49" s="5"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="11"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D50" s="1"/>
+      <c r="E50" s="35"/>
+      <c r="F50" s="47"/>
+      <c r="G50" s="47"/>
+      <c r="H50" s="5"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="11"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="5"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="11"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="18"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="5"/>
+    </row>
+    <row r="861" spans="10:10" x14ac:dyDescent="0.25">
+      <c r="J861" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1508,7 +1533,7 @@
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="7">
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D47:E47"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="A5:E5"/>
@@ -1517,11 +1542,11 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.78740157480314965" bottom="0.78740157480314965" header="0" footer="0"/>
+  <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <ignoredErrors>
-    <ignoredError sqref="E35:E37" unlockedFormula="1"/>
+    <ignoredError sqref="E39:E41" unlockedFormula="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactorizacion: centralize HTML component rendering with new config.render_html helper
</commit_message>
<xml_diff>
--- a/DOCS/REMITO_Master.xlsx
+++ b/DOCS/REMITO_Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORKS\CAPELLO SOMBREROS\APPLICATION\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7C1231-3F4B-458A-932A-42835517CB50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6DC6AB-3B06-40AD-B095-4B33F8D00803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="1140" windowWidth="21600" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Remito" sheetId="1" r:id="rId1"/>
@@ -80,9 +80,6 @@
     <t>vendidos</t>
   </si>
   <si>
-    <t>Observaciones</t>
-  </si>
-  <si>
     <t>Consignacion</t>
   </si>
   <si>
@@ -105,6 +102,9 @@
   </si>
   <si>
     <t>Capello</t>
+  </si>
+  <si>
+    <t>Resúmen</t>
   </si>
 </sst>
 </file>
@@ -856,11 +856,11 @@
     </row>
     <row r="2" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="1.05">
       <c r="A2" s="52" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2"/>
       <c r="C2" s="53" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2" s="54"/>
       <c r="E2" s="54"/>
@@ -926,7 +926,7 @@
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="66" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="67"/>
       <c r="C8" s="67"/>
@@ -935,7 +935,7 @@
       <c r="F8" s="67"/>
       <c r="G8" s="67"/>
       <c r="H8" s="50" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -955,13 +955,13 @@
         <v>12</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G9" s="27" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="I9" s="21"/>
       <c r="Q9" s="2"/>
@@ -1370,7 +1370,7 @@
     <row r="39" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A39" s="19"/>
       <c r="C39" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D39" s="5"/>
       <c r="E39" s="40">
@@ -1383,7 +1383,7 @@
       <c r="A40" s="11"/>
       <c r="B40" s="18"/>
       <c r="C40" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D40" s="5"/>
       <c r="E40" s="40">
@@ -1396,7 +1396,7 @@
       <c r="A41" s="11"/>
       <c r="B41" s="18"/>
       <c r="C41" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D41" s="5"/>
       <c r="E41" s="40">

</xml_diff>